<commit_message>
Add docx dependency for document export functionality and enhance schedule management with new export template dialog. Update database schema to include isTheoryCumPractical field for subjects, and modify relevant components and API routes to support this feature. Update test data files for subjects accordingly.
</commit_message>
<xml_diff>
--- a/test-data/subjects-sem1.xlsx
+++ b/test-data/subjects-sem1.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,6 +418,9 @@
       <c r="F1" t="str">
         <v>electiveGroupId</v>
       </c>
+      <c r="G1" t="str">
+        <v>tcp</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -438,6 +441,9 @@
       <c r="F2" t="str">
         <v/>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -458,6 +464,9 @@
       <c r="F3" t="str">
         <v/>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -478,6 +487,9 @@
       <c r="F4" t="str">
         <v/>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -498,6 +510,9 @@
       <c r="F5" t="str">
         <v/>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -518,6 +533,9 @@
       <c r="F6" t="str">
         <v/>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -538,10 +556,13 @@
       <c r="F7" t="str">
         <v/>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>